<commit_message>
mudancas nos graficos das tefs
</commit_message>
<xml_diff>
--- a/202505_resultados/tabelas_rmse_tefm/REQM_TFT_2022.xlsx
+++ b/202505_resultados/tabelas_rmse_tefm/REQM_TFT_2022.xlsx
@@ -422,37 +422,37 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>0,2125</t>
+          <t>0.2125</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0,0012</t>
+          <t>0.0012</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0,0012</t>
+          <t>0.0012</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0,0021</t>
+          <t>0.0021</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>0,0023</t>
+          <t>0.0023</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>0,0022</t>
+          <t>0.0022</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>0,0022</t>
+          <t>0.0022</t>
         </is>
       </c>
     </row>
@@ -469,37 +469,37 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>0,2127</t>
+          <t>0.2127</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>0,0008</t>
+          <t>0.0008</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>0,0008</t>
+          <t>0.0008</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>0,0019</t>
+          <t>0.0019</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>0,0020</t>
+          <t>0.0020</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>0,0020</t>
+          <t>0.0020</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>0,0020</t>
+          <t>0.0020</t>
         </is>
       </c>
     </row>
@@ -516,37 +516,37 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>0,2101</t>
+          <t>0.2101</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>0,0019</t>
+          <t>0.0019</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>0,0019</t>
+          <t>0.0019</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>0,0010</t>
+          <t>0.0010</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>0,0010</t>
+          <t>0.0010</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>0,0009</t>
+          <t>0.0009</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>0,0009</t>
+          <t>0.0009</t>
         </is>
       </c>
     </row>
@@ -563,37 +563,37 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>0,4242</t>
+          <t>0.4242</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>0,0018</t>
+          <t>0.0018</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>0,0018</t>
+          <t>0.0018</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>0,0041</t>
+          <t>0.0041</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>0,0044</t>
+          <t>0.0044</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>0,0043</t>
+          <t>0.0043</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>0,0043</t>
+          <t>0.0043</t>
         </is>
       </c>
     </row>
@@ -610,37 +610,37 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>0,4254</t>
+          <t>0.4254</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0,0016</t>
+          <t>0.0016</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>0,0016</t>
+          <t>0.0016</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>0,0039</t>
+          <t>0.0039</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>0,0041</t>
+          <t>0.0041</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>0,0039</t>
+          <t>0.0039</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>0,0040</t>
+          <t>0.0040</t>
         </is>
       </c>
     </row>
@@ -657,37 +657,37 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>0,4253</t>
+          <t>0.4253</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>0,0035</t>
+          <t>0.0035</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>0,0035</t>
+          <t>0.0035</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>0,0008</t>
+          <t>0.0008</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>0,0009</t>
+          <t>0.0009</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>0,0009</t>
+          <t>0.0009</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>0,0010</t>
+          <t>0.0010</t>
         </is>
       </c>
     </row>
@@ -704,37 +704,37 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>0,6346</t>
+          <t>0.6346</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0,0015</t>
+          <t>0.0015</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>0,0015</t>
+          <t>0.0015</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>0,0059</t>
+          <t>0.0059</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>0,0065</t>
+          <t>0.0065</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>0,0064</t>
+          <t>0.0064</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>0,0065</t>
+          <t>0.0065</t>
         </is>
       </c>
     </row>
@@ -751,37 +751,37 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>0,6379</t>
+          <t>0.6379</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0,0023</t>
+          <t>0.0023</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>0,0023</t>
+          <t>0.0023</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>0,0058</t>
+          <t>0.0058</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>0,0063</t>
+          <t>0.0063</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>0,0060</t>
+          <t>0.0060</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>0,0061</t>
+          <t>0.0061</t>
         </is>
       </c>
     </row>
@@ -798,37 +798,37 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>0,6377</t>
+          <t>0.6377</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0,0127</t>
+          <t>0.0127</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>0,0127</t>
+          <t>0.0127</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>0,0004</t>
+          <t>0.0004</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>0,0006</t>
+          <t>0.0006</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>0,0005</t>
+          <t>0.0005</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>0,0007</t>
+          <t>0.0007</t>
         </is>
       </c>
     </row>
@@ -845,37 +845,37 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>0,8462</t>
+          <t>0.8462</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0,0038</t>
+          <t>0.0038</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>0,0115</t>
+          <t>0.0115</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>0,0080</t>
+          <t>0.0080</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>0,0092</t>
+          <t>0.0092</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>0,0092</t>
+          <t>0.0092</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>0,0095</t>
+          <t>0.0095</t>
         </is>
       </c>
     </row>
@@ -892,37 +892,37 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>0,8507</t>
+          <t>0.8507</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0,0031</t>
+          <t>0.0031</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>0,0031</t>
+          <t>0.0031</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>0,0078</t>
+          <t>0.0078</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>0,0088</t>
+          <t>0.0088</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>0,0082</t>
+          <t>0.0082</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>0,0085</t>
+          <t>0.0085</t>
         </is>
       </c>
     </row>
@@ -939,37 +939,37 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0,8469</t>
+          <t>0.8469</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>0,0137</t>
+          <t>0.0137</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>0,0137</t>
+          <t>0.0137</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>0,0017</t>
+          <t>0.0017</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>0,0013</t>
+          <t>0.0013</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>0,0014</t>
+          <t>0.0014</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>0,0010</t>
+          <t>0.0010</t>
         </is>
       </c>
     </row>

</xml_diff>